<commit_message>
patch: new modules, time award, card refresh
</commit_message>
<xml_diff>
--- a/docs/数值分析_模块怪物波次.xlsx
+++ b/docs/数值分析_模块怪物波次.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -575,7 +575,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>26；波26仅 Boss HP=10000；Boss漏家即败</t>
+          <t>26；波26仅 Boss HP=50000；移速0.375；Boss漏家即败</t>
         </is>
       </c>
     </row>
@@ -606,10 +606,22 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
+          <t>窗口化</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1440×900；全屏=桌面分辨率</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>奥数飞弹</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>稀有；能耗1/容5/射速5；伤10/20/30/50/80；最右索敌</t>
         </is>
@@ -626,7 +638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -684,7 +696,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>10000</v>
+        <v>50000</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -695,205 +707,271 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>开局沙 ms</t>
+          <t>Boss 移速</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>100000</v>
+        <v>0.375</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>沙尽即败</t>
+          <t>坦克0.75的一半；单位格/秒</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>抽沙</t>
+          <t>红/黄/蓝移速</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>1000 ms/秒</t>
+          <t>1.5 / 3.0 / 0.75</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>仅战斗</t>
+          <t>紫拆·金盾同蓝</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>补沙</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>仅沙buff击杀</t>
-        </is>
+          <t>开局沙 ms</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>100000</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>清波不补沙</t>
+          <t>沙尽即败</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>手牌/商店</t>
+          <t>抽沙</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>8 / 6</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr"/>
+          <t>1000 ms/秒</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>仅战斗</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>商店池上限</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>12</v>
+          <t>补沙</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>仅沙buff击杀</t>
+        </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>开局：激光+收束+雪花+火花</t>
+          <t>清波不补沙</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>球上限</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>40</v>
+          <t>手牌/商店</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>8 / 6</t>
+        </is>
       </c>
       <c r="C10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>球寿命档</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>12/20/32/50 s</t>
-        </is>
+          <t>商店池上限</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>12</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>熔炉寿命维</t>
+          <t>开局：激光+收束+雪花+火花</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>分解返还</t>
+          <t>球上限</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>invested×30%</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>扩展费用</t>
+          <t>球寿命档</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>100 / 300</t>
+          <t>12/20/32/50 s</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>3→5 / 5→7</t>
+          <t>熔炉寿命维</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>刷新费</t>
+          <t>窗口化</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>5×((shopLv+1)/2)</t>
+          <t>1440×900</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>商店 Lv1–2→5，Lv3–4→10…</t>
+          <t>全屏=桌面分辨率</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>商店等级</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>(wave-1)//5+1</t>
-        </is>
+          <t>分解返还</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0.3</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>每5波升1级；奇级单档/偶级双档</t>
+          <t>invested×30%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>模块解锁</t>
+          <t>扩展费用</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>前15每3波，后每2波</t>
+          <t>100 / 300</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>3/6/9/12/16/18/20/22/24</t>
+          <t>3→5 / 5→7</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>刷新费</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>5×((shopLv+1)/2)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>商店 Lv1–2→5，Lv3–4→10…</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>商店等级</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>(wave-1)//5+1</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>每5波升1级；奇级单档/偶级双档</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>模块解锁</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>前15每3波，后每2波</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>3/6/9/12/16/18/20/22/24</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>熔炉/祝福</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>每5波至25</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>5/10/15/20/25</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>胜负</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>返回主菜单</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>ResultOverlay</t>
         </is>
       </c>
     </row>
@@ -5461,14 +5539,14 @@
       <c r="G27" s="3" t="inlineStr"/>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Boss 10000</t>
+          <t>Boss 50000</t>
         </is>
       </c>
       <c r="I27" s="3" t="n">
-        <v>10000</v>
+        <v>50000</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>-0.826</v>
+        <v>-0.132</v>
       </c>
       <c r="K27" s="3" t="n">
         <v>1905</v>

</xml_diff>